<commit_message>
noooot really sure what's goin on
</commit_message>
<xml_diff>
--- a/data/species_june_classified.xlsx
+++ b/data/species_june_classified.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30306"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B76CF1D2-0CAF-4B6C-B4FE-48C5D1405893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F091C21-DC1F-476F-AB1C-AD7218DE3A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -989,7 +989,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -1125,7 +1125,7 @@
         <v>65</v>
       </c>
       <c r="B62" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:2">

</xml_diff>